<commit_message>
Cria primeira versão do novo volume pdf/T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_base_legal_demonstrativos.xlsx
+++ b/bancos/manual/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\2.Programação e Normas\2023\PPAG 2023 e LOA 2023\Volumes\Demonstrativos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\volumes-loa\bancos\manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0109EFDD-06D7-4D09-B34D-15123BD54272}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEEDD893-3A64-4D50-B955-E42D0DB822A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="133">
   <si>
     <t>cod</t>
   </si>
@@ -432,13 +432,22 @@
   </si>
   <si>
     <t>(Art. 7º, Inciso XXIV da Lei 24.404/2023- LDO</t>
+  </si>
+  <si>
+    <t>T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO</t>
+  </si>
+  <si>
+    <t>39. Demonstrativo De Recursos A Serem Aplicados Direta Ou Indiretamente Em Ações Voltadas A Políticas De Atendimento À Mulher</t>
+  </si>
+  <si>
+    <t>(Art. X Inciso Y da Lei Z)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,15 +838,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="1" max="1" width="102.7109375" customWidth="1"/>
+    <col min="2" max="2" width="103.28515625" customWidth="1"/>
     <col min="3" max="3" width="167.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -848,7 +857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -859,7 +868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -870,7 +879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -881,7 +890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -892,7 +901,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -903,7 +912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -914,7 +923,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -925,7 +934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -936,7 +945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -947,7 +956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -958,7 +967,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -969,7 +978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -980,7 +989,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -991,7 +1000,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1002,7 +1011,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1013,7 +1022,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1024,7 +1033,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1035,7 +1044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1046,7 +1055,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30.75">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1057,7 +1066,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1079,7 +1088,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1090,7 +1099,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -1101,7 +1110,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1112,7 +1121,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>72</v>
       </c>
@@ -1123,7 +1132,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1134,7 +1143,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -1145,7 +1154,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -1154,6 +1163,17 @@
       </c>
       <c r="C29" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1165,14 +1185,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9730DD9-C36A-40E7-998B-E00A0695F1C5}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65.5703125" customWidth="1"/>
     <col min="2" max="2" width="33.140625" customWidth="1"/>
     <col min="3" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>82</v>
       </c>
@@ -1198,7 +1218,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30.75">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>90</v>
       </c>
@@ -1209,7 +1229,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30.75">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1220,7 +1240,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30.75">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -1231,7 +1251,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30.75">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1242,7 +1262,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30.75">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1253,7 +1273,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1264,7 +1284,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30.75">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -1275,7 +1295,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30.75">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -1286,7 +1306,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30.75">
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
@@ -1297,7 +1317,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30.75">
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>97</v>
       </c>
@@ -1308,7 +1328,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30.75">
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>99</v>
       </c>
@@ -1319,7 +1339,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1330,7 +1350,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30.75">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
@@ -1341,7 +1361,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30.75">
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1352,7 +1372,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30.75">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -1363,7 +1383,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60.75">
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1374,7 +1394,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="45.75">
+    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1405,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="45.75">
+    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
@@ -1396,7 +1416,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="45.75">
+    <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -1407,7 +1427,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="45.75">
+    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>49</v>
       </c>
@@ -1418,7 +1438,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30.75">
+    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>105</v>
       </c>
@@ -1429,7 +1449,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="37.5">
+    <row r="23" spans="1:8" ht="36" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>107</v>
       </c>
@@ -1440,7 +1460,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30.75">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>52</v>
       </c>
@@ -1451,7 +1471,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30.75">
+    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>110</v>
       </c>
@@ -1462,7 +1482,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="60.75">
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>55</v>
       </c>
@@ -1473,7 +1493,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30.75">
+    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -1485,7 +1505,7 @@
       </c>
       <c r="D27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="30.75">
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>61</v>
       </c>
@@ -1496,7 +1516,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30.75">
+    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>64</v>
       </c>
@@ -1507,7 +1527,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="30.75">
+    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>67</v>
       </c>
@@ -1518,7 +1538,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30.75">
+    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>116</v>
       </c>
@@ -1529,7 +1549,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>118</v>
       </c>
@@ -1540,7 +1560,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30.75">
+    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -1551,7 +1571,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>73</v>
       </c>
@@ -1562,7 +1582,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>76</v>
       </c>
@@ -1573,7 +1593,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>78</v>
       </c>
@@ -1584,7 +1604,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>122</v>
       </c>
@@ -1595,7 +1615,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>123</v>
       </c>
@@ -1606,7 +1626,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="30.75">
+    <row r="39" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>80</v>
       </c>
@@ -1617,7 +1637,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="37.5">
+    <row r="40" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>126</v>
       </c>
@@ -1628,7 +1648,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="30.75">
+    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>128</v>
       </c>
@@ -1645,6 +1665,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="18" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1b889f39a240c2e855286b20cf95d05e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="902f44b668f40cdc6ccc2fe791adf365" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -1899,7 +1928,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -1918,23 +1947,40 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Demonstrativo T39 - Política de Atendimento às Mulheres Vítimas de Violência no Estado (#120)
* Cria primeira versão do novo volume pdf/T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO

* Corrige nome da coluna  DR/IR no demonstrativo T39

* remove linhas comentadas do demonstrativo T39

* Altera script T39 para utilizar a base acoes_planejamento com a nova coluna 'acoes para mulheres'

* Cria teste e adiciona assets para o T39

* adiciona .tex do T39 para testes

---------

Co-authored-by: Francisco Júnior <fjunior.alves.oliveira@gmail.com>
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_base_legal_demonstrativos.xlsx
+++ b/bancos/manual/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\2.Programação e Normas\2023\PPAG 2023 e LOA 2023\Volumes\Demonstrativos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\volumes-loa\bancos\manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0109EFDD-06D7-4D09-B34D-15123BD54272}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEEDD893-3A64-4D50-B955-E42D0DB822A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="133">
   <si>
     <t>cod</t>
   </si>
@@ -432,13 +432,22 @@
   </si>
   <si>
     <t>(Art. 7º, Inciso XXIV da Lei 24.404/2023- LDO</t>
+  </si>
+  <si>
+    <t>T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO</t>
+  </si>
+  <si>
+    <t>39. Demonstrativo De Recursos A Serem Aplicados Direta Ou Indiretamente Em Ações Voltadas A Políticas De Atendimento À Mulher</t>
+  </si>
+  <si>
+    <t>(Art. X Inciso Y da Lei Z)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,15 +838,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="1" max="1" width="102.7109375" customWidth="1"/>
+    <col min="2" max="2" width="103.28515625" customWidth="1"/>
     <col min="3" max="3" width="167.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -848,7 +857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -859,7 +868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -870,7 +879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -881,7 +890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -892,7 +901,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -903,7 +912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -914,7 +923,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -925,7 +934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -936,7 +945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -947,7 +956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -958,7 +967,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -969,7 +978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -980,7 +989,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -991,7 +1000,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1002,7 +1011,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1013,7 +1022,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1024,7 +1033,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1035,7 +1044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1046,7 +1055,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30.75">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1057,7 +1066,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1079,7 +1088,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1090,7 +1099,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -1101,7 +1110,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1112,7 +1121,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>72</v>
       </c>
@@ -1123,7 +1132,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1134,7 +1143,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -1145,7 +1154,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -1154,6 +1163,17 @@
       </c>
       <c r="C29" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1165,14 +1185,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9730DD9-C36A-40E7-998B-E00A0695F1C5}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65.5703125" customWidth="1"/>
     <col min="2" max="2" width="33.140625" customWidth="1"/>
     <col min="3" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>82</v>
       </c>
@@ -1198,7 +1218,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30.75">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>90</v>
       </c>
@@ -1209,7 +1229,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30.75">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1220,7 +1240,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30.75">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -1231,7 +1251,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30.75">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1242,7 +1262,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30.75">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1253,7 +1273,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1264,7 +1284,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30.75">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -1275,7 +1295,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30.75">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -1286,7 +1306,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30.75">
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
@@ -1297,7 +1317,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30.75">
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>97</v>
       </c>
@@ -1308,7 +1328,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30.75">
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>99</v>
       </c>
@@ -1319,7 +1339,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1330,7 +1350,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30.75">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
@@ -1341,7 +1361,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30.75">
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1352,7 +1372,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30.75">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -1363,7 +1383,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60.75">
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1374,7 +1394,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="45.75">
+    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1405,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="45.75">
+    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
@@ -1396,7 +1416,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="45.75">
+    <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -1407,7 +1427,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="45.75">
+    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>49</v>
       </c>
@@ -1418,7 +1438,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30.75">
+    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>105</v>
       </c>
@@ -1429,7 +1449,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="37.5">
+    <row r="23" spans="1:8" ht="36" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>107</v>
       </c>
@@ -1440,7 +1460,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30.75">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>52</v>
       </c>
@@ -1451,7 +1471,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30.75">
+    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>110</v>
       </c>
@@ -1462,7 +1482,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="60.75">
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>55</v>
       </c>
@@ -1473,7 +1493,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30.75">
+    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -1485,7 +1505,7 @@
       </c>
       <c r="D27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="30.75">
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>61</v>
       </c>
@@ -1496,7 +1516,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30.75">
+    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>64</v>
       </c>
@@ -1507,7 +1527,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="30.75">
+    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>67</v>
       </c>
@@ -1518,7 +1538,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30.75">
+    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>116</v>
       </c>
@@ -1529,7 +1549,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>118</v>
       </c>
@@ -1540,7 +1560,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30.75">
+    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -1551,7 +1571,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>73</v>
       </c>
@@ -1562,7 +1582,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>76</v>
       </c>
@@ -1573,7 +1593,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>78</v>
       </c>
@@ -1584,7 +1604,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>122</v>
       </c>
@@ -1595,7 +1615,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>123</v>
       </c>
@@ -1606,7 +1626,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="30.75">
+    <row r="39" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>80</v>
       </c>
@@ -1617,7 +1637,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="37.5">
+    <row r="40" spans="1:6" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>126</v>
       </c>
@@ -1628,7 +1648,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="30.75">
+    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>128</v>
       </c>
@@ -1645,6 +1665,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="18" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1b889f39a240c2e855286b20cf95d05e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="902f44b668f40cdc6ccc2fe791adf365" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -1899,7 +1928,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -1918,23 +1947,40 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
make rm vol=4 && make v4
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_base_legal_demonstrativos.xlsx
+++ b/bancos/manual/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27318"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\volumes-loa\bancos\manual\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\2.Programação e Normas\2023\PPAG 2023 e LOA 2023\Volumes\Demonstrativos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEEDD893-3A64-4D50-B955-E42D0DB822A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0109EFDD-06D7-4D09-B34D-15123BD54272}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="130">
   <si>
     <t>cod</t>
   </si>
@@ -432,22 +432,13 @@
   </si>
   <si>
     <t>(Art. 7º, Inciso XXIV da Lei 24.404/2023- LDO</t>
-  </si>
-  <si>
-    <t>T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO</t>
-  </si>
-  <si>
-    <t>39. Demonstrativo De Recursos A Serem Aplicados Direta Ou Indiretamente Em Ações Voltadas A Políticas De Atendimento À Mulher</t>
-  </si>
-  <si>
-    <t>(Art. X Inciso Y da Lei Z)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -838,15 +829,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="102.7109375" customWidth="1"/>
-    <col min="2" max="2" width="103.28515625" customWidth="1"/>
+    <col min="1" max="1" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="167.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -857,7 +848,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -868,7 +859,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -879,7 +870,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -890,7 +881,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -901,7 +892,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -912,7 +903,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -923,7 +914,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -934,7 +925,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -945,7 +936,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -956,7 +947,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -967,7 +958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -978,7 +969,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -989,7 +980,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1000,7 +991,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1011,7 +1002,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1022,7 +1013,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1033,7 +1024,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1044,7 +1035,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1055,7 +1046,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="30.75">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1066,7 +1057,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1077,7 +1068,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1088,7 +1079,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1099,7 +1090,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -1110,7 +1101,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1121,7 +1112,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>72</v>
       </c>
@@ -1132,7 +1123,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1143,7 +1134,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -1154,7 +1145,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -1163,17 +1154,6 @@
       </c>
       <c r="C29" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>130</v>
-      </c>
-      <c r="B30" t="s">
-        <v>131</v>
-      </c>
-      <c r="C30" t="s">
-        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1185,14 +1165,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9730DD9-C36A-40E7-998B-E00A0695F1C5}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="65.5703125" customWidth="1"/>
     <col min="2" max="2" width="33.140625" customWidth="1"/>
     <col min="3" max="8" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>82</v>
       </c>
@@ -1218,7 +1198,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30.75">
       <c r="A2" s="3" t="s">
         <v>90</v>
       </c>
@@ -1229,7 +1209,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="30.75">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1240,7 +1220,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="30.75">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -1251,7 +1231,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="30.75">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1262,7 +1242,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="30.75">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1273,7 +1253,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1284,7 +1264,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="30.75">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -1295,7 +1275,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="30.75">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -1306,7 +1286,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="30.75">
       <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
@@ -1317,7 +1297,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="30.75">
       <c r="A11" s="8" t="s">
         <v>97</v>
       </c>
@@ -1328,7 +1308,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="30.75">
       <c r="A12" s="3" t="s">
         <v>99</v>
       </c>
@@ -1339,7 +1319,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1350,7 +1330,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="30.75">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
@@ -1361,7 +1341,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="30.75">
       <c r="A15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1372,7 +1352,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="30.75">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -1383,7 +1363,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="60.75">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1394,7 +1374,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="45.75">
       <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
@@ -1405,7 +1385,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="45.75">
       <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
@@ -1416,7 +1396,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="45.75">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -1427,7 +1407,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="45.75">
       <c r="A21" s="3" t="s">
         <v>49</v>
       </c>
@@ -1438,7 +1418,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="30.75">
       <c r="A22" s="8" t="s">
         <v>105</v>
       </c>
@@ -1449,7 +1429,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="37.5">
       <c r="A23" s="8" t="s">
         <v>107</v>
       </c>
@@ -1460,7 +1440,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="30.75">
       <c r="A24" s="8" t="s">
         <v>52</v>
       </c>
@@ -1471,7 +1451,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="30.75">
       <c r="A25" s="8" t="s">
         <v>110</v>
       </c>
@@ -1482,7 +1462,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="60.75">
       <c r="A26" s="3" t="s">
         <v>55</v>
       </c>
@@ -1493,7 +1473,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="30.75">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -1505,7 +1485,7 @@
       </c>
       <c r="D27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="30.75">
       <c r="A28" s="3" t="s">
         <v>61</v>
       </c>
@@ -1516,7 +1496,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="30.75">
       <c r="A29" s="3" t="s">
         <v>64</v>
       </c>
@@ -1527,7 +1507,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="30.75">
       <c r="A30" s="3" t="s">
         <v>67</v>
       </c>
@@ -1538,7 +1518,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="30.75">
       <c r="A31" s="8" t="s">
         <v>116</v>
       </c>
@@ -1549,7 +1529,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8">
       <c r="A32" s="8" t="s">
         <v>118</v>
       </c>
@@ -1560,7 +1540,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="30.75">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -1571,7 +1551,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="A34" s="3" t="s">
         <v>73</v>
       </c>
@@ -1582,7 +1562,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
         <v>76</v>
       </c>
@@ -1593,7 +1573,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
         <v>78</v>
       </c>
@@ -1604,7 +1584,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6">
       <c r="A37" s="8" t="s">
         <v>122</v>
       </c>
@@ -1615,7 +1595,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6">
       <c r="A38" s="8" t="s">
         <v>123</v>
       </c>
@@ -1626,7 +1606,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="36" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="30.75">
       <c r="A39" s="2" t="s">
         <v>80</v>
       </c>
@@ -1637,7 +1617,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="36" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="37.5">
       <c r="A40" s="8" t="s">
         <v>126</v>
       </c>
@@ -1648,7 +1628,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="30.75">
       <c r="A41" s="8" t="s">
         <v>128</v>
       </c>
@@ -1665,15 +1645,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="18" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1b889f39a240c2e855286b20cf95d05e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="902f44b668f40cdc6ccc2fe791adf365" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -1928,7 +1899,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -1947,40 +1918,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}"/>
 </file>
</xml_diff>

<commit_message>
make rm vol=1 && make v1
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_base_legal_demonstrativos.xlsx
+++ b/bancos/manual/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\2.Programação e Normas\2023\PPAG 2023 e LOA 2023\Volumes\Demonstrativos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fjunior/Projects/splor/volumes-loa/bancos/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0109EFDD-06D7-4D09-B34D-15123BD54272}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E5AE12-FDC2-0142-BAAF-0C53B48E037E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="133">
   <si>
     <t>cod</t>
   </si>
@@ -432,13 +432,22 @@
   </si>
   <si>
     <t>(Art. 7º, Inciso XXIV da Lei 24.404/2023- LDO</t>
+  </si>
+  <si>
+    <t>T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO</t>
+  </si>
+  <si>
+    <t>39. Demonstrativo Mulher</t>
+  </si>
+  <si>
+    <t>(Art XXX, foo)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,15 +838,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
-    <col min="3" max="3" width="167.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="167.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -848,7 +857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -859,7 +868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -870,7 +879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -881,7 +890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -892,7 +901,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -903,7 +912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -914,7 +923,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -925,7 +934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -936,7 +945,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -947,7 +956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -958,7 +967,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -969,7 +978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -980,7 +989,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -991,7 +1000,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1002,7 +1011,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1013,7 +1022,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1024,7 +1033,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1035,7 +1044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1046,7 +1055,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30.75">
+    <row r="20" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1057,7 +1066,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1068,7 +1077,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1079,7 +1088,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1090,7 +1099,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -1101,7 +1110,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1112,7 +1121,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>72</v>
       </c>
@@ -1123,7 +1132,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1134,7 +1143,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -1145,7 +1154,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -1154,6 +1163,17 @@
       </c>
       <c r="C29" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1165,14 +1185,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9730DD9-C36A-40E7-998B-E00A0695F1C5}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="65.5703125" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
-    <col min="3" max="8" width="9.140625" style="6"/>
+    <col min="1" max="1" width="65.5" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" customWidth="1"/>
+    <col min="3" max="8" width="9.1640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>82</v>
       </c>
@@ -1198,7 +1218,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30.75">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>90</v>
       </c>
@@ -1209,7 +1229,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30.75">
+    <row r="3" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1220,7 +1240,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30.75">
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -1231,7 +1251,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30.75">
+    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1242,7 +1262,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30.75">
+    <row r="6" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
@@ -1253,7 +1273,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1264,7 +1284,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30.75">
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -1275,7 +1295,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30.75">
+    <row r="9" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -1286,7 +1306,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30.75">
+    <row r="10" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>25</v>
       </c>
@@ -1297,7 +1317,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30.75">
+    <row r="11" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>97</v>
       </c>
@@ -1308,7 +1328,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30.75">
+    <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>99</v>
       </c>
@@ -1319,7 +1339,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1330,7 +1350,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30.75">
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
@@ -1341,7 +1361,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30.75">
+    <row r="15" spans="1:8" ht="26" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>33</v>
       </c>
@@ -1352,7 +1372,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30.75">
+    <row r="16" spans="1:8" ht="26" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -1363,7 +1383,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60.75">
+    <row r="17" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1374,7 +1394,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="45.75">
+    <row r="18" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1405,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="45.75">
+    <row r="19" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
@@ -1396,7 +1416,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="45.75">
+    <row r="20" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -1407,7 +1427,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="45.75">
+    <row r="21" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>49</v>
       </c>
@@ -1418,7 +1438,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30.75">
+    <row r="22" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>105</v>
       </c>
@@ -1429,7 +1449,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="37.5">
+    <row r="23" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>107</v>
       </c>
@@ -1440,7 +1460,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30.75">
+    <row r="24" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>52</v>
       </c>
@@ -1451,7 +1471,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30.75">
+    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>110</v>
       </c>
@@ -1462,7 +1482,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="60.75">
+    <row r="26" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>55</v>
       </c>
@@ -1473,7 +1493,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="30.75">
+    <row r="27" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>58</v>
       </c>
@@ -1485,7 +1505,7 @@
       </c>
       <c r="D27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="30.75">
+    <row r="28" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>61</v>
       </c>
@@ -1496,7 +1516,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="30.75">
+    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>64</v>
       </c>
@@ -1507,7 +1527,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="30.75">
+    <row r="30" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>67</v>
       </c>
@@ -1518,7 +1538,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="30.75">
+    <row r="31" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>116</v>
       </c>
@@ -1529,7 +1549,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
         <v>118</v>
       </c>
@@ -1540,7 +1560,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30.75">
+    <row r="33" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -1551,7 +1571,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>73</v>
       </c>
@@ -1562,7 +1582,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>76</v>
       </c>
@@ -1573,7 +1593,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>78</v>
       </c>
@@ -1584,7 +1604,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>122</v>
       </c>
@@ -1595,7 +1615,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
         <v>123</v>
       </c>
@@ -1606,7 +1626,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="30.75">
+    <row r="39" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>80</v>
       </c>
@@ -1617,7 +1637,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="37.5">
+    <row r="40" spans="1:6" ht="39" x14ac:dyDescent="0.2">
       <c r="A40" s="8" t="s">
         <v>126</v>
       </c>
@@ -1628,7 +1648,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="30.75">
+    <row r="41" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="8" t="s">
         <v>128</v>
       </c>
@@ -1900,6 +1920,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -1918,23 +1947,40 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C048F50-7DE2-4464-BD5C-A1BECFD191AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FF4EF5B-0E3B-4873-A6D2-6087C9EC9166}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FCAB9D5-4699-48C8-8DB7-84FDCD7CDA0C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(ploa): alterações e geração dos volumes 2ª iteração.
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_base_legal_demonstrativos.xlsx
+++ b/bancos/manual/desc_base_legal_demonstrativos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/DCPPN 2026/PPAG e LOA 2026/PPAG/material de apoio - gerar volumes/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/DCPPN 2026/PPAG e LOA 2026/material de apoio/material de apoio - gerar volumes/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="404" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8601CC6-C21C-4811-ABA2-F524E54DC065}"/>
+  <xr:revisionPtr revIDLastSave="416" documentId="11_A3DD8646BA7476893AAB1FDD9F017BEA3498940F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AABACC1-D64D-48C7-8AD2-BF49F9BB0DE6}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_legal" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="136">
   <si>
     <t>cod</t>
   </si>
@@ -60,9 +60,6 @@
     <t>02. Demonstrativo da Receita Corrente Fiscal</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XXII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T3_DCGF_Demonstrativo_Receita_Despesa_Segundo_Categorias_Economicas</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>05. Demonstrativo Consolidado da Categoria de Pessoal por Unidade Orçamentária</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XXIII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T6_DCGF_Demonstrativo_Evolucao_Receita_por_Categoria_Economica</t>
   </si>
   <si>
@@ -114,18 +108,12 @@
     <t>08. Demonstrativo da Receita Corrente Líquida</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso II da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T9_DEMONSTRATIVO_RECEITA_ORCAMENTARIA_CORRENTE_ORDINARIA</t>
   </si>
   <si>
     <t>09. Demonstrativo da Receita Orçamentária Corrente Ordinária</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XV da Lei 24.945/2024 -  LDO)</t>
-  </si>
-  <si>
     <t>T12_DCGF_Demonstrativo_Evolucao_Despesa_Categoria_Economica</t>
   </si>
   <si>
@@ -159,100 +147,66 @@
     <t>16. Demonstrativo da Aplicação de Recursos na Manutenção e no Desenvolvimento do Ensino</t>
   </si>
   <si>
-    <t>(Art. 212 da Constituição Federal, Art. 201 da Constituição Estadual e Art. 7º, Inciso III da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T17_DCGF_Demonst_Aplicacao_Recursos_Progr_Saude_Investim</t>
   </si>
   <si>
     <t>17. Demonstrativo da Aplicação de Recursos em Programas de Saúde e em Investimentos em Transporte e Sistema Viário</t>
   </si>
   <si>
-    <t>(Art. 158,  §1º da Constituição Estadual e Art. 7º, Inciso IV da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T18_DCGF_Demonst_Aplicacao_Recursos_Acoes_Servicos_Publicos_Saude</t>
   </si>
   <si>
     <t>18. Demonstrativo da Aplicação de Recursos em Ações e Serviços Públicos de Saúde</t>
   </si>
   <si>
-    <t>(Art. 198 da Constituição Federal e Art. 7°, Inciso V da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T19_DCGF_Demonstrativo_Aplicacao_Recursos_Amparo_Fomento_Pesquisa</t>
   </si>
   <si>
     <t>19. Demonstrativo da Aplicação de Recursos no Amparo e Fomento à Pesquisa</t>
   </si>
   <si>
-    <t>(Art. 212 da Constituição Estadual e Art. 7°, Inciso VI da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T20A_DCGF_Demonstrativo_Partic_Percentual_Pessoal_RCL_LRF</t>
   </si>
   <si>
     <t>20. Demonstrativo da Participação Percentual de Pessoal na Receita Corrente Líquida</t>
   </si>
   <si>
-    <t>(Art. 19 da Lei Complementar 101/2000 - LRF e Art. 7°, Inciso VIII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T23_DCGF_Demonstrativo_do_Servico_da_divida_publica</t>
   </si>
   <si>
     <t>23. Demonstrativo do Serviço da Dívida Pública</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XIII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T25_DCGF_Demonstrativo_Aplicacao_Recursos_FUNDEB</t>
   </si>
   <si>
     <t>25. Demonstrativo da Aplicação dos Recursos do Fundo de Desenvolvimento da Educação Básica e Valorização dos Profissionais da Educação</t>
   </si>
   <si>
-    <t xml:space="preserve">(Art. 212-A da Constituição Federal, Art. 60 do ADCT/CF e Art. 7°, Inciso XII
-da Lei 24.945/2024 - LDO)                                                                                                                                               </t>
-  </si>
-  <si>
     <t>T26_DCGF_DEMONSTRATIVO_RECURSOS_APLICADOS_ACOES_PARA_CRIANCA_E_ADOLESCENTE</t>
   </si>
   <si>
     <t>26.  Demonstrativo dos recursos a serem aplicados, direta ou indiretamente, em ações voltadas para a criança e o adolescente</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XVIII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T27_DCGF_Demonst_Despesas_UGEPREVI</t>
   </si>
   <si>
     <t>27. Demonstrativo  das  despesas  da  Unidade  de  Gestão Previdenciária  Integrada  -  UGEPREVI</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso X da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T38_DCGF_DEMONSTRATIVO_RECEITAS_DESPESAS_PREVIDENCIARIAS_RPPS</t>
   </si>
   <si>
     <t>28. Demonstrativo das Receitas e Despesas Previdenciárias</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XI da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T28_DCGF</t>
   </si>
   <si>
     <t>29. Demonstrativo dos programas financiados com recursos provenientes da União</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XX da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T30_INVESTIMENTOS_SEGUNDO_FUNCOES</t>
   </si>
   <si>
@@ -268,18 +222,12 @@
     <t>34. Investimentos Segundo Funções, Subfunções e Programas por Projetos e Atividades</t>
   </si>
   <si>
-    <t>(Art. 31 da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T32_INVESTIMENTOS_POR_EMPRESA_SEGUNDO_FONTES_RECURSO</t>
   </si>
   <si>
     <t>35. Investimentos por Empresas Segundo Fonte de Recurso</t>
   </si>
   <si>
-    <t>(Art. 32 da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T33_INVESTIMENTOS_EMPRESA_SEGUNDO_DETALHAMENTO_INVESTIMENTOS</t>
   </si>
   <si>
@@ -292,16 +240,10 @@
     <t>39.    Demonstrativo dos recursos a serem aplicados, direta ou indiretamente, na  execução  da  Política  Estadual  de Segurança Alimentar e Nutricional Sustentável - PESANS</t>
   </si>
   <si>
-    <t>(Art. 7º, Inciso XVII da Lei 24.945/2024 - LDO)</t>
-  </si>
-  <si>
     <t>T39_DCGF_DEMONSTRATIVO_DA_POLITICA_DE_ATENDIMENTO_A_MULHER_VITIMA_DE_VIOLENCIA_NO_ESTADO</t>
   </si>
   <si>
     <t>34. Demonstrativo dos recursos a serem aplicados, direta ou indiretamente, na execução da política de atendimento à mulher vítima de violência no Estado, conforme o disposto na Lei nº 22.256, de 26 de julho de 2016.</t>
-  </si>
-  <si>
-    <t>(Art. 7º, Inciso XXV da Lei 24.945/2024 - LDO)</t>
   </si>
   <si>
     <t>DEMONSTRATIVOS CONSOLIDADOS DO ORÇAMENTO FISCAL</t>
@@ -1057,6 +999,7 @@
           <cell r="C27" t="str">
             <v>x</v>
           </cell>
+          <cell r="D27"/>
           <cell r="I27" t="str">
             <v>carolina</v>
           </cell>
@@ -1141,6 +1084,7 @@
           <cell r="C33" t="str">
             <v>x</v>
           </cell>
+          <cell r="D33"/>
           <cell r="I33" t="str">
             <v>Izabella</v>
           </cell>
@@ -1608,315 +1552,315 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="B30" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1940,48 +1884,48 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="K1" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP(A2,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -1993,10 +1937,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I3" t="str">
         <f>VLOOKUP(A3,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2005,13 +1949,13 @@
     </row>
     <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E4" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I4" t="str">
         <f>VLOOKUP(A4,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2020,41 +1964,41 @@
     </row>
     <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="C5" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I5" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I6" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I7" t="str">
         <f>VLOOKUP(A7,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2063,13 +2007,13 @@
     </row>
     <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I8" t="str">
         <f>VLOOKUP(A8,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2078,13 +2022,13 @@
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I9" t="str">
         <f>VLOOKUP(A9,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2093,13 +2037,13 @@
     </row>
     <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I10" t="str">
         <f>VLOOKUP(A10,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2108,13 +2052,13 @@
     </row>
     <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I11" t="str">
         <f>VLOOKUP(A11,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2123,13 +2067,13 @@
     </row>
     <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I12" t="str">
         <f>VLOOKUP(A12,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2138,13 +2082,13 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I13" t="str">
         <f>VLOOKUP(A13,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2153,13 +2097,13 @@
     </row>
     <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I14" t="str">
         <f>VLOOKUP(A14,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2168,41 +2112,41 @@
     </row>
     <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I15" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I16" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I17" t="str">
         <f>VLOOKUP(A17,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2211,13 +2155,13 @@
     </row>
     <row r="18" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I18" t="str">
         <f>VLOOKUP(A18,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2226,13 +2170,13 @@
     </row>
     <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I19" t="str">
         <f>VLOOKUP(A19,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2241,13 +2185,13 @@
     </row>
     <row r="20" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I20" t="str">
         <f>VLOOKUP(A20,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2256,13 +2200,13 @@
     </row>
     <row r="21" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I21" t="str">
         <f>VLOOKUP(A21,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2271,13 +2215,13 @@
     </row>
     <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I22" t="str">
         <f>VLOOKUP(A22,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2286,13 +2230,13 @@
     </row>
     <row r="23" spans="1:9" ht="36" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I23" t="str">
         <f>VLOOKUP(A23,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2301,13 +2245,13 @@
     </row>
     <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I24" t="str">
         <f>VLOOKUP(A24,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2316,13 +2260,13 @@
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I25" t="str">
         <f>VLOOKUP(A25,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2331,13 +2275,13 @@
     </row>
     <row r="26" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I26" t="str">
         <f>VLOOKUP(A26,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2346,13 +2290,13 @@
     </row>
     <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D27" s="7"/>
       <c r="I27" t="str">
@@ -2362,13 +2306,13 @@
     </row>
     <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I28" t="str">
         <f>VLOOKUP(A28,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2377,13 +2321,13 @@
     </row>
     <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I29" t="str">
         <f>VLOOKUP(A29,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2392,13 +2336,13 @@
     </row>
     <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I30" t="str">
         <f>VLOOKUP(A30,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2407,13 +2351,13 @@
     </row>
     <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I31" t="str">
         <f>VLOOKUP(A31,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2422,13 +2366,13 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I32" t="str">
         <f>VLOOKUP(A32,'[1]Controle de conferencia LOA'!A$2:I$47,9,FALSE)</f>
@@ -2437,206 +2381,206 @@
     </row>
     <row r="33" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I33" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I34" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I35" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I36" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I37" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I38" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I39" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="36" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I40" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="36" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I41" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="I42" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="I43" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="I44" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="I45" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="I46" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="I47" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="I48" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="I49" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="I50" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>